<commit_message>
Sync planning SharePoint : S13
</commit_message>
<xml_diff>
--- a/Plannings 2026 S13.xlsx
+++ b/Plannings 2026 S13.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29905"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cdalpes.sharepoint.com/sites/msteams_bd0f90/Documents partages/02. USP - TOS - General/RH/Plannings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="24" documentId="8_{CF1412DF-E0EE-4DF3-9F8E-B4DFB4486AFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C73050A3-D4D5-4E23-A41B-81DFF0DAEEA1}"/>
+  <xr:revisionPtr revIDLastSave="36" documentId="8_{CF1412DF-E0EE-4DF3-9F8E-B4DFB4486AFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{05A02A9F-6A10-418F-80FB-C7CA5EEA7B0F}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -455,7 +455,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[h]:mm"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -795,7 +795,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -935,18 +935,6 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -956,16 +944,34 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -4339,6 +4345,490 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>74</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>74</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="82" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000052000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>76</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>76</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="83" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000053000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>78</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>78</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="84" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000054000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>80</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>80</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="85" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000055000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>82</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>82</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="86" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000056000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>82</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>82</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="87" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000057000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>84</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>84</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="88" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000058000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>74</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>74</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="89" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FA2E640D-B466-413A-B992-4D80C79981CD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1828800" y="12763500"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>76</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>76</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="90" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{85C830B4-DB6E-4FF6-8290-6568775E70A6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="17879786" y="14790964"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="91" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{70625FC7-9785-48DF-9CDC-DA58A6A7D317}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8939893" y="9756321"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="92" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A40EA93B-103B-4685-BDC7-F2B3C0854475}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8939893" y="3524250"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
       <xdr:col>6</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>74</xdr:row>
@@ -4352,10 +4842,54 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="80" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000050000000}"/>
+        <xdr:cNvPr id="93" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E780A7C6-4B58-475D-A7E5-E5101DDF4872}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="17879786" y="12464143"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>76</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>76</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="94" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7F1D2C41-CAE9-4D0D-A4CB-19E28EE62ECF}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4371,7 +4905,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="0"/>
+          <a:off x="17879786" y="12845143"/>
           <a:ext cx="123825" cy="123825"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4385,21 +4919,65 @@
     <xdr:from>
       <xdr:col>6</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>76</xdr:row>
+      <xdr:row>64</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>76</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="81" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000051000000}"/>
+      <xdr:row>64</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="95" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{714EF945-FD4A-4E9D-991E-15DDE07D3A8C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="14899821" y="14409964"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="96" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D568FE09-D35E-4F76-9494-EDFAEBB31A65}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4415,491 +4993,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="123825" cy="123825"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>74</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>74</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="82" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000052000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="123825" cy="123825"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>76</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>76</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="83" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000053000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="123825" cy="123825"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>78</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>78</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="84" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000054000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="123825" cy="123825"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>80</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>80</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="85" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000055000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="123825" cy="123825"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>82</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>82</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="86" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000056000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="123825" cy="123825"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>82</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>82</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="87" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000057000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="123825" cy="123825"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>84</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>84</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="88" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000058000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="123825" cy="123825"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>74</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>74</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="89" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FA2E640D-B466-413A-B992-4D80C79981CD}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1828800" y="12763500"/>
-          <a:ext cx="123825" cy="123825"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>76</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>76</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="90" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{85C830B4-DB6E-4FF6-8290-6568775E70A6}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="17879786" y="14790964"/>
-          <a:ext cx="123825" cy="123825"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>50</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>50</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="91" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{70625FC7-9785-48DF-9CDC-DA58A6A7D317}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="8939893" y="9756321"/>
-          <a:ext cx="123825" cy="123825"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="92" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A40EA93B-103B-4685-BDC7-F2B3C0854475}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="8939893" y="3524250"/>
+          <a:off x="14899821" y="14790964"/>
           <a:ext cx="123825" cy="123825"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4959,6 +5053,10 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5282,34 +5380,34 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:H87"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="8" width="44.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
-      <c r="B1" s="47" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="47"/>
-      <c r="D1" s="47"/>
-      <c r="E1" s="47"/>
-      <c r="F1" s="47"/>
-      <c r="G1" s="47"/>
-      <c r="H1" s="47"/>
-    </row>
-    <row r="2" spans="1:8">
-      <c r="B2" s="47" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B1" s="55" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="55"/>
+      <c r="D1" s="55"/>
+      <c r="E1" s="55"/>
+      <c r="F1" s="55"/>
+      <c r="G1" s="55"/>
+      <c r="H1" s="55"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B2" s="55" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="47"/>
-      <c r="D2" s="47"/>
-      <c r="E2" s="47"/>
-      <c r="F2" s="47"/>
-      <c r="G2" s="47"/>
-      <c r="H2" s="47"/>
-    </row>
-    <row r="3" spans="1:8">
+      <c r="C2" s="55"/>
+      <c r="D2" s="55"/>
+      <c r="E2" s="55"/>
+      <c r="F2" s="55"/>
+      <c r="G2" s="55"/>
+      <c r="H2" s="55"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
         <v>2</v>
       </c>
@@ -5332,7 +5430,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="15.75" thickBot="1">
+    <row r="4" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="12" t="s">
         <v>8</v>
       </c>
@@ -5358,8 +5456,8 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:8">
-      <c r="A5" s="48" t="s">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="50" t="s">
         <v>16</v>
       </c>
       <c r="B5" s="14"/>
@@ -5372,8 +5470,8 @@
       </c>
       <c r="H5" s="7"/>
     </row>
-    <row r="6" spans="1:8" ht="15.75" thickBot="1">
-      <c r="A6" s="49"/>
+    <row r="6" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="52"/>
       <c r="B6" s="15"/>
       <c r="C6" s="8"/>
       <c r="D6" s="8"/>
@@ -5384,20 +5482,20 @@
       </c>
       <c r="H6" s="9"/>
     </row>
-    <row r="7" spans="1:8" ht="15.75" thickBot="1">
+    <row r="7" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="51"/>
-      <c r="C7" s="52"/>
-      <c r="D7" s="52"/>
-      <c r="E7" s="52"/>
-      <c r="F7" s="52"/>
-      <c r="G7" s="52"/>
-      <c r="H7" s="53"/>
-    </row>
-    <row r="8" spans="1:8">
-      <c r="A8" s="48" t="s">
+      <c r="B7" s="47"/>
+      <c r="C7" s="48"/>
+      <c r="D7" s="48"/>
+      <c r="E7" s="48"/>
+      <c r="F7" s="48"/>
+      <c r="G7" s="48"/>
+      <c r="H7" s="49"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="50" t="s">
         <v>20</v>
       </c>
       <c r="B8" s="6" t="s">
@@ -5420,8 +5518,8 @@
       </c>
       <c r="H8" s="7"/>
     </row>
-    <row r="9" spans="1:8">
-      <c r="A9" s="50"/>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="51"/>
       <c r="B9" s="2" t="s">
         <v>25</v>
       </c>
@@ -5442,8 +5540,8 @@
       </c>
       <c r="H9" s="10"/>
     </row>
-    <row r="10" spans="1:8">
-      <c r="A10" s="50"/>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="51"/>
       <c r="B10" s="22" t="s">
         <v>22</v>
       </c>
@@ -5458,8 +5556,8 @@
       </c>
       <c r="H10" s="10"/>
     </row>
-    <row r="11" spans="1:8" ht="15.75" thickBot="1">
-      <c r="A11" s="49"/>
+    <row r="11" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="52"/>
       <c r="B11" s="21" t="s">
         <v>31</v>
       </c>
@@ -5474,8 +5572,8 @@
       </c>
       <c r="H11" s="9"/>
     </row>
-    <row r="12" spans="1:8">
-      <c r="A12" s="48" t="s">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="50" t="s">
         <v>34</v>
       </c>
       <c r="B12" s="6"/>
@@ -5488,8 +5586,8 @@
       <c r="G12" s="6"/>
       <c r="H12" s="7"/>
     </row>
-    <row r="13" spans="1:8" ht="15.75" thickBot="1">
-      <c r="A13" s="49"/>
+    <row r="13" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="52"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8" t="s">
         <v>35</v>
@@ -5500,20 +5598,20 @@
       <c r="G13" s="8"/>
       <c r="H13" s="9"/>
     </row>
-    <row r="14" spans="1:8" ht="15.75" thickBot="1">
+    <row r="14" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="B14" s="51"/>
-      <c r="C14" s="52"/>
-      <c r="D14" s="52"/>
-      <c r="E14" s="52"/>
-      <c r="F14" s="52"/>
-      <c r="G14" s="52"/>
-      <c r="H14" s="53"/>
-    </row>
-    <row r="15" spans="1:8">
-      <c r="A15" s="48" t="s">
+      <c r="B14" s="47"/>
+      <c r="C14" s="48"/>
+      <c r="D14" s="48"/>
+      <c r="E14" s="48"/>
+      <c r="F14" s="48"/>
+      <c r="G14" s="48"/>
+      <c r="H14" s="49"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="50" t="s">
         <v>37</v>
       </c>
       <c r="B15" s="6"/>
@@ -5530,8 +5628,8 @@
       </c>
       <c r="H15" s="7"/>
     </row>
-    <row r="16" spans="1:8" ht="15.75" thickBot="1">
-      <c r="A16" s="49"/>
+    <row r="16" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="52"/>
       <c r="B16" s="8"/>
       <c r="C16" s="8"/>
       <c r="D16" s="8" t="s">
@@ -5546,8 +5644,8 @@
       </c>
       <c r="H16" s="9"/>
     </row>
-    <row r="17" spans="1:8">
-      <c r="A17" s="48" t="s">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="50" t="s">
         <v>39</v>
       </c>
       <c r="B17" s="27" t="s">
@@ -5568,8 +5666,8 @@
         <v>21</v>
       </c>
     </row>
-    <row r="18" spans="1:8">
-      <c r="A18" s="50"/>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="51"/>
       <c r="B18" s="28" t="s">
         <v>42</v>
       </c>
@@ -5588,8 +5686,8 @@
         <v>46</v>
       </c>
     </row>
-    <row r="19" spans="1:8">
-      <c r="A19" s="50"/>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="51"/>
       <c r="B19" s="3" t="s">
         <v>47</v>
       </c>
@@ -5606,8 +5704,8 @@
         <v>40</v>
       </c>
     </row>
-    <row r="20" spans="1:8">
-      <c r="A20" s="50"/>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="51"/>
       <c r="B20" s="2" t="s">
         <v>48</v>
       </c>
@@ -5624,8 +5722,8 @@
         <v>51</v>
       </c>
     </row>
-    <row r="21" spans="1:8">
-      <c r="A21" s="50"/>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" s="51"/>
       <c r="B21" s="19" t="s">
         <v>40</v>
       </c>
@@ -5640,8 +5738,8 @@
       <c r="G21" s="2"/>
       <c r="H21" s="40"/>
     </row>
-    <row r="22" spans="1:8">
-      <c r="A22" s="50"/>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" s="51"/>
       <c r="B22" s="18" t="s">
         <v>52</v>
       </c>
@@ -5656,8 +5754,8 @@
       <c r="G22" s="2"/>
       <c r="H22" s="40"/>
     </row>
-    <row r="23" spans="1:8">
-      <c r="A23" s="50"/>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" s="51"/>
       <c r="B23" s="18"/>
       <c r="C23" s="3" t="s">
         <v>47</v>
@@ -5670,8 +5768,8 @@
       <c r="G23" s="2"/>
       <c r="H23" s="40"/>
     </row>
-    <row r="24" spans="1:8">
-      <c r="A24" s="50"/>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" s="51"/>
       <c r="B24" s="18"/>
       <c r="C24" s="2" t="s">
         <v>55</v>
@@ -5684,8 +5782,8 @@
       <c r="G24" s="2"/>
       <c r="H24" s="40"/>
     </row>
-    <row r="25" spans="1:8">
-      <c r="A25" s="50"/>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" s="51"/>
       <c r="B25" s="18"/>
       <c r="C25" s="19" t="s">
         <v>40</v>
@@ -5696,8 +5794,8 @@
       <c r="G25" s="2"/>
       <c r="H25" s="40"/>
     </row>
-    <row r="26" spans="1:8" ht="15.75" thickBot="1">
-      <c r="A26" s="49"/>
+    <row r="26" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="52"/>
       <c r="B26" s="17"/>
       <c r="C26" s="17" t="s">
         <v>52</v>
@@ -5708,8 +5806,8 @@
       <c r="G26" s="8"/>
       <c r="H26" s="41"/>
     </row>
-    <row r="27" spans="1:8">
-      <c r="A27" s="48" t="s">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" s="50" t="s">
         <v>57</v>
       </c>
       <c r="B27" s="6"/>
@@ -5722,8 +5820,8 @@
       </c>
       <c r="H27" s="7"/>
     </row>
-    <row r="28" spans="1:8" ht="15.75" thickBot="1">
-      <c r="A28" s="49"/>
+    <row r="28" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="52"/>
       <c r="B28" s="8"/>
       <c r="C28" s="8"/>
       <c r="D28" s="8"/>
@@ -5734,8 +5832,8 @@
       </c>
       <c r="H28" s="9"/>
     </row>
-    <row r="29" spans="1:8">
-      <c r="A29" s="48" t="s">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" s="50" t="s">
         <v>58</v>
       </c>
       <c r="B29" s="16" t="s">
@@ -5754,8 +5852,8 @@
       <c r="G29" s="6"/>
       <c r="H29" s="7"/>
     </row>
-    <row r="30" spans="1:8">
-      <c r="A30" s="50"/>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" s="51"/>
       <c r="B30" s="18" t="s">
         <v>60</v>
       </c>
@@ -5772,8 +5870,8 @@
       <c r="G30" s="2"/>
       <c r="H30" s="10"/>
     </row>
-    <row r="31" spans="1:8">
-      <c r="A31" s="50"/>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" s="51"/>
       <c r="B31" s="22" t="s">
         <v>64</v>
       </c>
@@ -5790,8 +5888,8 @@
       <c r="G31" s="2"/>
       <c r="H31" s="10"/>
     </row>
-    <row r="32" spans="1:8">
-      <c r="A32" s="50"/>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" s="51"/>
       <c r="B32" s="20" t="s">
         <v>65</v>
       </c>
@@ -5808,8 +5906,8 @@
       <c r="G32" s="2"/>
       <c r="H32" s="10"/>
     </row>
-    <row r="33" spans="1:8">
-      <c r="A33" s="50"/>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" s="51"/>
       <c r="B33" s="20"/>
       <c r="C33" s="3" t="s">
         <v>21</v>
@@ -5824,8 +5922,8 @@
       <c r="G33" s="2"/>
       <c r="H33" s="10"/>
     </row>
-    <row r="34" spans="1:8">
-      <c r="A34" s="50"/>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" s="51"/>
       <c r="B34" s="20"/>
       <c r="C34" s="2" t="s">
         <v>69</v>
@@ -5840,8 +5938,8 @@
       <c r="G34" s="2"/>
       <c r="H34" s="10"/>
     </row>
-    <row r="35" spans="1:8">
-      <c r="A35" s="50"/>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" s="51"/>
       <c r="B35" s="20"/>
       <c r="C35" s="2"/>
       <c r="D35" s="31" t="s">
@@ -5852,8 +5950,8 @@
       <c r="G35" s="2"/>
       <c r="H35" s="10"/>
     </row>
-    <row r="36" spans="1:8">
-      <c r="A36" s="50"/>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36" s="51"/>
       <c r="B36" s="20"/>
       <c r="C36" s="2"/>
       <c r="D36" s="30" t="s">
@@ -5864,8 +5962,8 @@
       <c r="G36" s="2"/>
       <c r="H36" s="10"/>
     </row>
-    <row r="37" spans="1:8">
-      <c r="A37" s="50"/>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37" s="51"/>
       <c r="B37" s="20"/>
       <c r="C37" s="2"/>
       <c r="D37" s="19" t="s">
@@ -5876,8 +5974,8 @@
       <c r="G37" s="2"/>
       <c r="H37" s="10"/>
     </row>
-    <row r="38" spans="1:8">
-      <c r="A38" s="50"/>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A38" s="51"/>
       <c r="B38" s="20"/>
       <c r="C38" s="2"/>
       <c r="D38" s="18" t="s">
@@ -5888,8 +5986,8 @@
       <c r="G38" s="2"/>
       <c r="H38" s="10"/>
     </row>
-    <row r="39" spans="1:8">
-      <c r="A39" s="50"/>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A39" s="51"/>
       <c r="B39" s="20"/>
       <c r="C39" s="2"/>
       <c r="D39" s="22" t="s">
@@ -5900,8 +5998,8 @@
       <c r="G39" s="2"/>
       <c r="H39" s="10"/>
     </row>
-    <row r="40" spans="1:8" ht="15.75" thickBot="1">
-      <c r="A40" s="49"/>
+    <row r="40" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="52"/>
       <c r="B40" s="21"/>
       <c r="C40" s="8"/>
       <c r="D40" s="21" t="s">
@@ -5912,32 +6010,32 @@
       <c r="G40" s="8"/>
       <c r="H40" s="9"/>
     </row>
-    <row r="41" spans="1:8" ht="15.75" thickBot="1">
+    <row r="41" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="B41" s="51"/>
-      <c r="C41" s="52"/>
-      <c r="D41" s="52"/>
-      <c r="E41" s="52"/>
-      <c r="F41" s="52"/>
-      <c r="G41" s="52"/>
-      <c r="H41" s="53"/>
-    </row>
-    <row r="42" spans="1:8" ht="15.75" thickBot="1">
+      <c r="B41" s="47"/>
+      <c r="C41" s="48"/>
+      <c r="D41" s="48"/>
+      <c r="E41" s="48"/>
+      <c r="F41" s="48"/>
+      <c r="G41" s="48"/>
+      <c r="H41" s="49"/>
+    </row>
+    <row r="42" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="13" t="s">
         <v>75</v>
       </c>
-      <c r="B42" s="51"/>
-      <c r="C42" s="52"/>
-      <c r="D42" s="52"/>
-      <c r="E42" s="52"/>
-      <c r="F42" s="52"/>
-      <c r="G42" s="52"/>
-      <c r="H42" s="53"/>
-    </row>
-    <row r="43" spans="1:8">
-      <c r="A43" s="48" t="s">
+      <c r="B42" s="47"/>
+      <c r="C42" s="48"/>
+      <c r="D42" s="48"/>
+      <c r="E42" s="48"/>
+      <c r="F42" s="48"/>
+      <c r="G42" s="48"/>
+      <c r="H42" s="49"/>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A43" s="50" t="s">
         <v>76</v>
       </c>
       <c r="B43" s="6"/>
@@ -5950,8 +6048,8 @@
         <v>21</v>
       </c>
     </row>
-    <row r="44" spans="1:8" ht="15.75" thickBot="1">
-      <c r="A44" s="49"/>
+    <row r="44" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="52"/>
       <c r="B44" s="8"/>
       <c r="C44" s="8"/>
       <c r="D44" s="8"/>
@@ -5962,20 +6060,20 @@
         <v>77</v>
       </c>
     </row>
-    <row r="45" spans="1:8" ht="15.75" thickBot="1">
+    <row r="45" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="13" t="s">
         <v>78</v>
       </c>
-      <c r="B45" s="51"/>
-      <c r="C45" s="52"/>
-      <c r="D45" s="52"/>
-      <c r="E45" s="52"/>
-      <c r="F45" s="52"/>
-      <c r="G45" s="52"/>
-      <c r="H45" s="53"/>
-    </row>
-    <row r="46" spans="1:8">
-      <c r="A46" s="48" t="s">
+      <c r="B45" s="47"/>
+      <c r="C45" s="48"/>
+      <c r="D45" s="48"/>
+      <c r="E45" s="48"/>
+      <c r="F45" s="48"/>
+      <c r="G45" s="48"/>
+      <c r="H45" s="49"/>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A46" s="50" t="s">
         <v>79</v>
       </c>
       <c r="B46" s="6"/>
@@ -5988,8 +6086,8 @@
       <c r="G46" s="6"/>
       <c r="H46" s="7"/>
     </row>
-    <row r="47" spans="1:8" ht="15.75" thickBot="1">
-      <c r="A47" s="49"/>
+    <row r="47" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="52"/>
       <c r="B47" s="8"/>
       <c r="C47" s="8"/>
       <c r="D47" s="8"/>
@@ -6000,20 +6098,20 @@
       <c r="G47" s="8"/>
       <c r="H47" s="9"/>
     </row>
-    <row r="48" spans="1:8" ht="15.75" thickBot="1">
+    <row r="48" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="B48" s="51"/>
-      <c r="C48" s="52"/>
-      <c r="D48" s="52"/>
-      <c r="E48" s="52"/>
-      <c r="F48" s="52"/>
-      <c r="G48" s="52"/>
-      <c r="H48" s="53"/>
-    </row>
-    <row r="49" spans="1:8">
-      <c r="A49" s="55" t="s">
+      <c r="B48" s="47"/>
+      <c r="C48" s="48"/>
+      <c r="D48" s="48"/>
+      <c r="E48" s="48"/>
+      <c r="F48" s="48"/>
+      <c r="G48" s="48"/>
+      <c r="H48" s="49"/>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A49" s="53" t="s">
         <v>81</v>
       </c>
       <c r="B49" s="20" t="s">
@@ -6030,8 +6128,8 @@
       <c r="G49" s="2"/>
       <c r="H49" s="10"/>
     </row>
-    <row r="50" spans="1:8" ht="15.75" thickBot="1">
-      <c r="A50" s="49"/>
+    <row r="50" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="52"/>
       <c r="B50" s="21" t="s">
         <v>73</v>
       </c>
@@ -6046,8 +6144,8 @@
       <c r="G50" s="8"/>
       <c r="H50" s="9"/>
     </row>
-    <row r="51" spans="1:8">
-      <c r="A51" s="48" t="s">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A51" s="50" t="s">
         <v>84</v>
       </c>
       <c r="B51" s="6" t="s">
@@ -6068,8 +6166,8 @@
       </c>
       <c r="H51" s="7"/>
     </row>
-    <row r="52" spans="1:8">
-      <c r="A52" s="50"/>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A52" s="51"/>
       <c r="B52" s="2" t="s">
         <v>85</v>
       </c>
@@ -6088,8 +6186,8 @@
       </c>
       <c r="H52" s="10"/>
     </row>
-    <row r="53" spans="1:8">
-      <c r="A53" s="50"/>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A53" s="51"/>
       <c r="B53" s="2"/>
       <c r="C53" s="22" t="s">
         <v>64</v>
@@ -6102,8 +6200,8 @@
       </c>
       <c r="H53" s="10"/>
     </row>
-    <row r="54" spans="1:8">
-      <c r="A54" s="50"/>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A54" s="51"/>
       <c r="B54" s="2"/>
       <c r="C54" s="20" t="s">
         <v>73</v>
@@ -6116,8 +6214,8 @@
       </c>
       <c r="H54" s="10"/>
     </row>
-    <row r="55" spans="1:8">
-      <c r="A55" s="50"/>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A55" s="51"/>
       <c r="B55" s="2"/>
       <c r="C55" s="20"/>
       <c r="D55" s="2"/>
@@ -6128,8 +6226,8 @@
       </c>
       <c r="H55" s="10"/>
     </row>
-    <row r="56" spans="1:8">
-      <c r="A56" s="50"/>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A56" s="51"/>
       <c r="B56" s="2"/>
       <c r="C56" s="20"/>
       <c r="D56" s="2"/>
@@ -6140,8 +6238,8 @@
       </c>
       <c r="H56" s="10"/>
     </row>
-    <row r="57" spans="1:8">
-      <c r="A57" s="50"/>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A57" s="51"/>
       <c r="B57" s="2"/>
       <c r="C57" s="20"/>
       <c r="D57" s="2"/>
@@ -6152,8 +6250,8 @@
       </c>
       <c r="H57" s="10"/>
     </row>
-    <row r="58" spans="1:8" ht="15.75" thickBot="1">
-      <c r="A58" s="49"/>
+    <row r="58" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="52"/>
       <c r="B58" s="8"/>
       <c r="C58" s="21"/>
       <c r="D58" s="8"/>
@@ -6164,8 +6262,8 @@
       </c>
       <c r="H58" s="9"/>
     </row>
-    <row r="59" spans="1:8">
-      <c r="A59" s="48" t="s">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A59" s="50" t="s">
         <v>91</v>
       </c>
       <c r="B59" s="6"/>
@@ -6180,8 +6278,8 @@
       <c r="G59" s="6"/>
       <c r="H59" s="7"/>
     </row>
-    <row r="60" spans="1:8" ht="15.75" thickBot="1">
-      <c r="A60" s="49"/>
+    <row r="60" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="52"/>
       <c r="B60" s="8"/>
       <c r="C60" s="17" t="s">
         <v>60</v>
@@ -6194,8 +6292,8 @@
       <c r="G60" s="8"/>
       <c r="H60" s="9"/>
     </row>
-    <row r="61" spans="1:8">
-      <c r="A61" s="48" t="s">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A61" s="50" t="s">
         <v>92</v>
       </c>
       <c r="B61" s="6" t="s">
@@ -6218,8 +6316,8 @@
         <v>93</v>
       </c>
     </row>
-    <row r="62" spans="1:8">
-      <c r="A62" s="50"/>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A62" s="51"/>
       <c r="B62" s="2" t="s">
         <v>29</v>
       </c>
@@ -6240,8 +6338,8 @@
         <v>96</v>
       </c>
     </row>
-    <row r="63" spans="1:8">
-      <c r="A63" s="50"/>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A63" s="51"/>
       <c r="B63" s="3" t="s">
         <v>21</v>
       </c>
@@ -6254,8 +6352,8 @@
         <v>21</v>
       </c>
     </row>
-    <row r="64" spans="1:8" ht="15.75" thickBot="1">
-      <c r="A64" s="49"/>
+    <row r="64" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="52"/>
       <c r="B64" s="8" t="s">
         <v>97</v>
       </c>
@@ -6268,8 +6366,8 @@
         <v>98</v>
       </c>
     </row>
-    <row r="65" spans="1:8">
-      <c r="A65" s="48" t="s">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A65" s="50" t="s">
         <v>99</v>
       </c>
       <c r="B65" s="23" t="s">
@@ -6279,15 +6377,15 @@
       <c r="D65" s="6"/>
       <c r="E65" s="6"/>
       <c r="F65" s="6"/>
-      <c r="G65" s="6" t="s">
-        <v>21</v>
+      <c r="G65" s="38" t="s">
+        <v>89</v>
       </c>
       <c r="H65" s="34" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="66" spans="1:8">
-      <c r="A66" s="50"/>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A66" s="51"/>
       <c r="B66" s="20" t="s">
         <v>73</v>
       </c>
@@ -6295,43 +6393,43 @@
       <c r="D66" s="2"/>
       <c r="E66" s="2"/>
       <c r="F66" s="2"/>
-      <c r="G66" s="2" t="s">
-        <v>100</v>
+      <c r="G66" s="39" t="s">
+        <v>103</v>
       </c>
       <c r="H66" s="35" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="67" spans="1:8">
-      <c r="A67" s="50"/>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A67" s="51"/>
       <c r="B67" s="20"/>
       <c r="C67" s="2"/>
       <c r="D67" s="2"/>
       <c r="E67" s="2"/>
       <c r="F67" s="2"/>
-      <c r="G67" s="32" t="s">
-        <v>89</v>
+      <c r="G67" s="3" t="s">
+        <v>21</v>
       </c>
       <c r="H67" s="36" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="68" spans="1:8" ht="15.75" thickBot="1">
-      <c r="A68" s="49"/>
+    <row r="68" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A68" s="52"/>
       <c r="B68" s="21"/>
       <c r="C68" s="8"/>
       <c r="D68" s="8"/>
       <c r="E68" s="8"/>
       <c r="F68" s="8"/>
-      <c r="G68" s="33" t="s">
-        <v>102</v>
+      <c r="G68" s="2" t="s">
+        <v>52</v>
       </c>
       <c r="H68" s="37" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="69" spans="1:8">
-      <c r="A69" s="48" t="s">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A69" s="50" t="s">
         <v>104</v>
       </c>
       <c r="B69" s="6"/>
@@ -6346,8 +6444,8 @@
         <v>89</v>
       </c>
     </row>
-    <row r="70" spans="1:8" ht="15.75" thickBot="1">
-      <c r="A70" s="49"/>
+    <row r="70" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A70" s="52"/>
       <c r="B70" s="8"/>
       <c r="C70" s="8"/>
       <c r="D70" s="17" t="s">
@@ -6360,8 +6458,8 @@
         <v>106</v>
       </c>
     </row>
-    <row r="71" spans="1:8">
-      <c r="A71" s="48" t="s">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A71" s="50" t="s">
         <v>107</v>
       </c>
       <c r="B71" s="6"/>
@@ -6374,8 +6472,8 @@
       </c>
       <c r="H71" s="7"/>
     </row>
-    <row r="72" spans="1:8">
-      <c r="A72" s="50"/>
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A72" s="51"/>
       <c r="B72" s="2"/>
       <c r="C72" s="2"/>
       <c r="D72" s="2"/>
@@ -6386,8 +6484,8 @@
       </c>
       <c r="H72" s="10"/>
     </row>
-    <row r="73" spans="1:8">
-      <c r="A73" s="50"/>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A73" s="51"/>
       <c r="B73" s="2"/>
       <c r="C73" s="2"/>
       <c r="D73" s="2"/>
@@ -6398,8 +6496,8 @@
       </c>
       <c r="H73" s="10"/>
     </row>
-    <row r="74" spans="1:8" ht="15.75" thickBot="1">
-      <c r="A74" s="49"/>
+    <row r="74" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A74" s="52"/>
       <c r="B74" s="8"/>
       <c r="C74" s="8"/>
       <c r="D74" s="8"/>
@@ -6410,8 +6508,8 @@
       </c>
       <c r="H74" s="9"/>
     </row>
-    <row r="75" spans="1:8">
-      <c r="A75" s="48" t="s">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A75" s="50" t="s">
         <v>108</v>
       </c>
       <c r="B75" s="6"/>
@@ -6421,15 +6519,15 @@
       </c>
       <c r="E75" s="6"/>
       <c r="F75" s="6"/>
-      <c r="G75" s="38" t="s">
-        <v>89</v>
+      <c r="G75" s="6" t="s">
+        <v>21</v>
       </c>
       <c r="H75" s="7" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="76" spans="1:8">
-      <c r="A76" s="50"/>
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A76" s="51"/>
       <c r="B76" s="2"/>
       <c r="C76" s="2"/>
       <c r="D76" s="18" t="s">
@@ -6437,15 +6535,15 @@
       </c>
       <c r="E76" s="2"/>
       <c r="F76" s="2"/>
-      <c r="G76" s="39" t="s">
-        <v>103</v>
+      <c r="G76" s="2" t="s">
+        <v>100</v>
       </c>
       <c r="H76" s="10" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="77" spans="1:8">
-      <c r="A77" s="50"/>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A77" s="51"/>
       <c r="B77" s="2"/>
       <c r="C77" s="2"/>
       <c r="D77" s="3" t="s">
@@ -6453,15 +6551,15 @@
       </c>
       <c r="E77" s="2"/>
       <c r="F77" s="2"/>
-      <c r="G77" s="3" t="s">
-        <v>21</v>
+      <c r="G77" s="32" t="s">
+        <v>89</v>
       </c>
       <c r="H77" s="36" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="78" spans="1:8">
-      <c r="A78" s="50"/>
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A78" s="51"/>
       <c r="B78" s="2"/>
       <c r="C78" s="2"/>
       <c r="D78" s="2" t="s">
@@ -6469,63 +6567,63 @@
       </c>
       <c r="E78" s="2"/>
       <c r="F78" s="2"/>
-      <c r="G78" s="2" t="s">
-        <v>52</v>
+      <c r="G78" s="39" t="s">
+        <v>102</v>
       </c>
       <c r="H78" s="35" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="79" spans="1:8">
-      <c r="A79" s="50"/>
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A79" s="51"/>
       <c r="B79" s="2"/>
       <c r="C79" s="2"/>
       <c r="D79" s="2"/>
       <c r="E79" s="2"/>
       <c r="F79" s="2"/>
-      <c r="G79" s="2"/>
+      <c r="G79" s="58"/>
       <c r="H79" s="11" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="80" spans="1:8">
-      <c r="A80" s="50"/>
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A80" s="51"/>
       <c r="B80" s="2"/>
       <c r="C80" s="2"/>
       <c r="D80" s="2"/>
       <c r="E80" s="2"/>
       <c r="F80" s="2"/>
-      <c r="G80" s="2"/>
+      <c r="G80" s="58"/>
       <c r="H80" s="10" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="81" spans="1:8">
-      <c r="A81" s="50"/>
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A81" s="51"/>
       <c r="B81" s="2"/>
       <c r="C81" s="2"/>
       <c r="D81" s="2"/>
       <c r="E81" s="2"/>
       <c r="F81" s="2"/>
-      <c r="G81" s="2"/>
+      <c r="G81" s="58"/>
       <c r="H81" s="36" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="82" spans="1:8" ht="15.75" thickBot="1">
-      <c r="A82" s="49"/>
+    <row r="82" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A82" s="52"/>
       <c r="B82" s="8"/>
       <c r="C82" s="8"/>
       <c r="D82" s="8"/>
       <c r="E82" s="8"/>
       <c r="F82" s="8"/>
-      <c r="G82" s="8"/>
+      <c r="G82" s="59"/>
       <c r="H82" s="37" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="83" spans="1:8">
-      <c r="A83" s="48" t="s">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A83" s="50" t="s">
         <v>114</v>
       </c>
       <c r="B83" s="6" t="s">
@@ -6540,8 +6638,8 @@
       <c r="G83" s="6"/>
       <c r="H83" s="7"/>
     </row>
-    <row r="84" spans="1:8" ht="15.75" thickBot="1">
-      <c r="A84" s="49"/>
+    <row r="84" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A84" s="52"/>
       <c r="B84" s="8" t="s">
         <v>115</v>
       </c>
@@ -6554,8 +6652,8 @@
       <c r="G84" s="8"/>
       <c r="H84" s="9"/>
     </row>
-    <row r="85" spans="1:8">
-      <c r="A85" s="48" t="s">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A85" s="50" t="s">
         <v>117</v>
       </c>
       <c r="B85" s="6"/>
@@ -6568,8 +6666,8 @@
       <c r="G85" s="6"/>
       <c r="H85" s="7"/>
     </row>
-    <row r="86" spans="1:8" ht="15.75" thickBot="1">
-      <c r="A86" s="49"/>
+    <row r="86" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A86" s="52"/>
       <c r="B86" s="8"/>
       <c r="C86" s="8"/>
       <c r="D86" s="17" t="s">
@@ -6580,7 +6678,7 @@
       <c r="G86" s="8"/>
       <c r="H86" s="9"/>
     </row>
-    <row r="87" spans="1:8" ht="3.75" customHeight="1">
+    <row r="87" spans="1:8" ht="3.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B87" s="54"/>
       <c r="C87" s="54"/>
       <c r="D87" s="54"/>
@@ -6591,6 +6689,22 @@
     </row>
   </sheetData>
   <mergeCells count="28">
+    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="A8:A11"/>
+    <mergeCell ref="A46:A47"/>
+    <mergeCell ref="B41:H41"/>
+    <mergeCell ref="B42:H42"/>
+    <mergeCell ref="B45:H45"/>
+    <mergeCell ref="A83:A84"/>
+    <mergeCell ref="A85:A86"/>
+    <mergeCell ref="B87:H87"/>
+    <mergeCell ref="A51:A58"/>
+    <mergeCell ref="A59:A60"/>
+    <mergeCell ref="A61:A64"/>
+    <mergeCell ref="A65:A68"/>
+    <mergeCell ref="A69:A70"/>
     <mergeCell ref="B48:H48"/>
     <mergeCell ref="B7:H7"/>
     <mergeCell ref="B14:H14"/>
@@ -6603,22 +6717,6 @@
     <mergeCell ref="A15:A16"/>
     <mergeCell ref="A17:A26"/>
     <mergeCell ref="A27:A28"/>
-    <mergeCell ref="A83:A84"/>
-    <mergeCell ref="A85:A86"/>
-    <mergeCell ref="B87:H87"/>
-    <mergeCell ref="A51:A58"/>
-    <mergeCell ref="A59:A60"/>
-    <mergeCell ref="A61:A64"/>
-    <mergeCell ref="A65:A68"/>
-    <mergeCell ref="A69:A70"/>
-    <mergeCell ref="B2:H2"/>
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="A8:A11"/>
-    <mergeCell ref="A46:A47"/>
-    <mergeCell ref="B41:H41"/>
-    <mergeCell ref="B42:H42"/>
-    <mergeCell ref="B45:H45"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="36" fitToHeight="0" orientation="landscape" r:id="rId1"/>
@@ -6629,14 +6727,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E34"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75">
+    <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B4" s="56" t="s">
         <v>119</v>
       </c>
@@ -6644,7 +6742,7 @@
       <c r="D4" s="56"/>
       <c r="E4" s="56"/>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B5" s="57" t="s">
         <v>120</v>
       </c>
@@ -6652,7 +6750,7 @@
       <c r="D5" s="57"/>
       <c r="E5" s="57"/>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
@@ -6669,7 +6767,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="42" t="s">
         <v>16</v>
       </c>
@@ -6686,7 +6784,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="42" t="s">
         <v>19</v>
       </c>
@@ -6703,7 +6801,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="42" t="s">
         <v>20</v>
       </c>
@@ -6720,7 +6818,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="42" t="s">
         <v>34</v>
       </c>
@@ -6737,7 +6835,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="42" t="s">
         <v>36</v>
       </c>
@@ -6754,7 +6852,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="42" t="s">
         <v>37</v>
       </c>
@@ -6771,7 +6869,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="42" t="s">
         <v>39</v>
       </c>
@@ -6788,7 +6886,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:5">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="42" t="s">
         <v>57</v>
       </c>
@@ -6805,7 +6903,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:5">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="42" t="s">
         <v>58</v>
       </c>
@@ -6822,7 +6920,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:5">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="42" t="s">
         <v>74</v>
       </c>
@@ -6839,7 +6937,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:5">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="42" t="s">
         <v>125</v>
       </c>
@@ -6856,7 +6954,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:5">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="42" t="s">
         <v>75</v>
       </c>
@@ -6873,7 +6971,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="42" t="s">
         <v>76</v>
       </c>
@@ -6890,7 +6988,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="42" t="s">
         <v>78</v>
       </c>
@@ -6907,7 +7005,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:5">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="42" t="s">
         <v>79</v>
       </c>
@@ -6924,7 +7022,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:5">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="42" t="s">
         <v>126</v>
       </c>
@@ -6941,7 +7039,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:5">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="42" t="s">
         <v>80</v>
       </c>
@@ -6958,7 +7056,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:5">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="42" t="s">
         <v>81</v>
       </c>
@@ -6975,7 +7073,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:5">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="42" t="s">
         <v>84</v>
       </c>
@@ -6992,7 +7090,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:5">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="42" t="s">
         <v>91</v>
       </c>
@@ -7009,7 +7107,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:5">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="42" t="s">
         <v>92</v>
       </c>
@@ -7026,7 +7124,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:5">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="42" t="s">
         <v>99</v>
       </c>
@@ -7043,7 +7141,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:5">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="42" t="s">
         <v>104</v>
       </c>
@@ -7060,7 +7158,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:5">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="42" t="s">
         <v>107</v>
       </c>
@@ -7077,7 +7175,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:5">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="42" t="s">
         <v>108</v>
       </c>
@@ -7094,7 +7192,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:5">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="42" t="s">
         <v>114</v>
       </c>
@@ -7111,7 +7209,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:5">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="42" t="s">
         <v>117</v>
       </c>
@@ -7128,7 +7226,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:5">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B34" s="44">
         <v>0.16111200000000001</v>
       </c>
@@ -7154,14 +7252,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F22"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" ht="15.75">
+    <row r="1" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="45" t="s">
         <v>127</v>
       </c>
@@ -7169,13 +7267,13 @@
         <v>128</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="45" t="s">
         <v>129</v>
       </c>
       <c r="B5" s="46"/>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="45" t="s">
         <v>130</v>
       </c>
@@ -7183,7 +7281,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="45" t="s">
         <v>131</v>
       </c>
@@ -7191,7 +7289,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="45" t="s">
         <v>133</v>
       </c>
@@ -7199,7 +7297,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="22" spans="6:6">
+    <row r="22" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F22" t="s">
         <v>135</v>
       </c>
@@ -7356,15 +7454,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="3c298670-db79-47a5-968d-a4570c34317f">
@@ -7375,14 +7464,49 @@
 </p:properties>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{21EE6D31-AE7B-4F53-874C-4DA5173E9811}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{21EE6D31-AE7B-4F53-874C-4DA5173E9811}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="3c298670-db79-47a5-968d-a4570c34317f"/>
+    <ds:schemaRef ds:uri="17e8e7ea-beb0-4155-adc4-5bfa61f32508"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{448366C3-E961-448C-ACD4-00095B6C03BD}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B4EE930C-D754-4117-9097-6D7F83AAB916}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="3c298670-db79-47a5-968d-a4570c34317f"/>
+    <ds:schemaRef ds:uri="17e8e7ea-beb0-4155-adc4-5bfa61f32508"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B4EE930C-D754-4117-9097-6D7F83AAB916}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{448366C3-E961-448C-ACD4-00095B6C03BD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>